<commit_message>
SFV2: add 'Where to see it' (section + steps, real labels) to each Milos question
Per PO feedback: 'What happens now' had no anchor, so the PO couldn't tell where in
the app or via which steps the behaviour occurs. Each question now leads with a plain
'Where to see it' line (Settings > Work Orders tab; Parts > Purchase Orders) before the
behaviour and the question. xlsx + CSV both updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Po6jyqTxJVLHxQtwvT2Wv5
</commit_message>
<xml_diff>
--- a/build/simple-flow-v2/questions-2026-09-09/Simple Flow V2 - Questions for Milos Vasic.xlsx
+++ b/build/simple-flow-v2/questions-2026-09-09/Simple Flow V2 - Questions for Milos Vasic.xlsx
@@ -41,12 +41,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -85,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,13 +103,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -494,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>What is this?</t>
@@ -506,7 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>How to answer</t>
@@ -514,11 +525,11 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Open the tab for each question (Question 1, 2, 3 along the bottom). Read the short description, then type A or B in the yellow 'Your answer' box. Add a note if you want - totally optional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Open the tab for each question (Question 1, 2, 3 along the bottom). Each tab tells you WHERE in the app to look and WHAT to do to see it, then asks the question. Type A or B in the yellow 'Your answer' box; add a note if you like.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>In a hurry?</t>
@@ -530,7 +541,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No jargon</t>
@@ -538,11 +549,11 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Everything is in plain language - you don't need any technical detail to answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Everything is in plain language and uses the same button names you see in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Thank you</t>
@@ -550,7 +561,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>That's it. Your answers let us finish the tests correctly. Much appreciated!</t>
+          <t>Your answers let us finish the tests correctly. Much appreciated!</t>
         </is>
       </c>
     </row>
@@ -565,11 +576,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -582,77 +593,89 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+          <t>Read 'Where to see it' and 'What happens now', then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Where to see it</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Open the app's Settings and go to the 'Work Orders' tab (the page with on/off switches grouped under Workflow, Line Requirements and Parts, with a 'Save Settings' button at the bottom). Turn on or change several of these switches at the same time - for example 'Require Approval for New Lines' together with 'Require Ordering Parts' and 'Require Picking Inventory Parts' - then press 'Save Settings'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>What happens now</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>When an admin changes several of these settings together, the 'approval' setting is applied first. But changing 'approval' never changes any work that already exists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>When those switches are saved together, the 'approval' one is handled first. But turning approval on or off never changes any work order line that already exists - it only affects new lines from then on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>The question</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Does applying 'approval' first actually change anything - or does it simply mean that work still waiting for approval is skipped when the other settings are applied?</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Since approval never changes existing work, does handling it 'first' actually change anything - or does it simply mean that lines still waiting for approval are skipped when the other switches take effect?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Option A</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>A - It simply means work waiting for approval is skipped. Nothing else to check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>A - It simply means lines still awaiting approval are skipped. Nothing else to check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Option B</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>B - Applying it first does something else we should check. (Please tell us what, in Notes.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>B - Handling it first does something else we should check. (Please tell us what, in Notes.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>(type A or B here)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Notes (optional)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -665,94 +688,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The 'Select all' box on the receive list</t>
+          <t>The 'Select all' box on the Purchase Orders list</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+          <t>Read 'Where to see it' and 'What happens now', then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Where to see it</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>In the top menu open 'Parts', then click 'Purchase Orders' in the left sidebar (under Supply Chain). This is the list of purchase orders, each row with a 'Receive' button. The list shows about thirty rows and loads more as you scroll down. Now tick the 'select all' checkbox at the very top of the list (its header).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>What happens now</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>The receive list shows about thirty rows at a time and loads more as you scroll down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Ticking 'select all' selects only the rows currently loaded on screen (about thirty). Rows further down that haven't loaded yet are not selected - the bar then says something like '30 Purchase Orders selected'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>The question</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>When you press 'Select all', it ticks only the rows already on screen (about thirty) - not the ones further down. Is that okay for now?</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Is it okay for now that 'select all' selects only the ~30 rows already loaded, not every purchase order further down the list?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Option A</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>A - Yes, that's fine for now.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Option B</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>B - No, 'Select all' should tick every row. Please raise it as a problem to fix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>B - No, 'Select all' should select every purchase order. Please raise it as a problem to fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>(type A or B here)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Notes (optional)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -765,94 +800,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Very large changes</t>
+          <t>Very large changes to existing jobs</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Please read the two short boxes, then type A or B in the yellow box.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+          <t>Read 'Where to see it' and 'What happens now', then type A or B in the yellow box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
+          <t>Where to see it</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>In the app's Settings, on the same 'Work Orders' tab as Question 1, change one of the on/off switches and press 'Save Settings'. That change is applied to the work orders you already have. Try it once where only a few jobs are affected, and imagine (or set up) a case where a very large number of jobs are affected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>What happens now</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>A small change happens straight away on screen. A very large one runs quietly in the background, and the screen shows advice to make it after working hours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>A change that affects only a few jobs is applied straight away on screen. A change that affects a very large number of jobs runs quietly in the background instead, and the screen shows advice to make the change after working hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>The question</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>How many affected jobs count as 'too large to do on screen', and how many should trigger the 'do it after hours' advice? (An engineer may need to give the numbers.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>How many affected jobs should count as 'too large to do on screen' (so it runs in the background), and how many should trigger the 'do it after hours' advice? (An engineer may need to give the two numbers.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Option A</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>A - Here are the two numbers: ____ and ____ (type them in Notes).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Option B</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>B - Not decided yet - for now just check the wait affects only the admin who made the change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>B - Not decided yet - for now just check that the wait affects only the admin who made the change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>(type A or B here)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Notes (optional)</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -869,7 +916,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="88" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
@@ -884,67 +931,67 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Type A or B in each yellow box. Full detail is on the numbered tabs.</t>
+          <t>Each line says where in the app it is. Type A or B in the yellow box; full steps are on the numbered tabs.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>The question in one line</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>The question (and where to see it)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Your answer (A/B)</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="11" t="n">
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>When several settings change at once, does 'approval first' matter, or does it just skip work still awaiting approval?</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>In Settings &gt; 'Work Orders' tab: when you save several on/off switches at once, the 'approval' one is applied first but never changes existing lines. Does 'first' matter, or does it just mean lines still awaiting approval are skipped?</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr"/>
+      <c r="D5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Is it okay that 'Select all' ticks only the ~30 rows on screen, not the ones further down?</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="11" t="n">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>On Parts &gt; Purchase Orders (the receive list): 'Select all' ticks only the ~30 rows loaded on screen, not the ones further down. Okay for now?</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr"/>
+      <c r="D6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>What are the two size limits for 'runs in the background' and 'do it after hours' advice?</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr"/>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>In Settings &gt; 'Work Orders' tab: a change hitting a few jobs applies on screen; a very large one runs in the background with 'after hours' advice. What are the two size limits?</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr"/>
+      <c r="D7" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -961,9 +1008,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -981,88 +1028,88 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Q#</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Cases it decides</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Why it is a question, not a defect</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="5" ht="88" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>C44554 - https://shopview.testrail.io/index.php?/cases/view/44554</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Epic SV-8683 / Story SV-9248 (Story 2) / spec 771391574 (rev 8 Sep 2026), Story 2 Requirements</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Epic SV-8683 / Story SV-9248 (Story 2) / spec 771391574 (rev 8 Sep 2026), Story 2 Requirements; Settings &gt; Work Orders tab (Require Approval for New Lines, Require Ordering Parts, Require Picking Inventory Parts)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Spec says both 'approval applied first, then ordering, then picking' AND 'turning approval on/off changes no existing line'. If approval never sweeps, precedence is a no-op on existing data. C44554 item 5 tests only exclusion of not-yet-approved parts; precedence left unwritten pending Milos.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="6" ht="88" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>C53488 - https://shopview.testrail.io/index.php?/cases/view/53488</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Epic SV-8683 / Story SV-9260 (Story 14) / spec 771391574 (rev 8 Sep 2026), Story 14 receive page &amp; PO bulk receive</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Spec records paged Select-all (one page, ~30 rows) as EXPECTED, resolving when pagination is replaced - outside this release. Confirming keeps C53488 a Pass, not a raised deviation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Epic SV-8683 / Story SV-9260 (Story 14) / spec 771391574 (rev 8 Sep 2026); Parts &gt; Purchase Orders (/parts/orders), header select-all -&gt; 'N Purchase Orders selected'</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Spec records paged Select-all (one page, ~30 rows) as EXPECTED, resolving when pagination is replaced - outside this release. Confirming keeps C53488 a Pass, not a raised deviation. (Route confirmed on build 2026-09-09.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="88" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>C44559 - https://shopview.testrail.io/index.php?/cases/view/44559</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Epic SV-8683 / Story SV-9250 (Story 4) / spec 771391574 (rev 8 Sep 2026), Story 4 Applying at scale</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Epic SV-8683 / Story SV-9250 (Story 4) / spec 771391574 (rev 8 Sep 2026); Settings &gt; Work Orders tab, applying a setting change at scale</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Two volume thresholds (in-request vs background; off-hours advisory) are 'agreed with engineering', not stated. Admin-only-blocking is testable now (C44559); the two boundaries need concrete numbers.</t>
         </is>

</xml_diff>